<commit_message>
✨ feat: Adiciona novas instâncias e resultados associados
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m100000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -477,25 +477,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5.5</v>
+        <v>3.25</v>
       </c>
       <c r="D2" t="n">
-        <v>74</v>
+        <v>710</v>
       </c>
       <c r="E2" t="n">
-        <v>74</v>
+        <v>710</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>15.40377402305603</v>
+        <v>159.2079517841339</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m100000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -504,25 +504,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5.5</v>
+        <v>3.25</v>
       </c>
       <c r="D3" t="n">
-        <v>74</v>
+        <v>710</v>
       </c>
       <c r="E3" t="n">
-        <v>74</v>
+        <v>710</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>13.31495332717896</v>
+        <v>714.4901256561279</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m100000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -531,25 +531,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5.75</v>
+        <v>3.5</v>
       </c>
       <c r="D4" t="n">
-        <v>63</v>
+        <v>552</v>
       </c>
       <c r="E4" t="n">
-        <v>63</v>
+        <v>552</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>4.367571115493774</v>
+        <v>170.8507416248322</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m100000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -558,25 +558,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5.75</v>
+        <v>3.5</v>
       </c>
       <c r="D5" t="n">
-        <v>63</v>
+        <v>552</v>
       </c>
       <c r="E5" t="n">
-        <v>63</v>
+        <v>552</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>6.059481620788574</v>
+        <v>898.1498346328735</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m100000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -585,25 +585,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6</v>
+        <v>3.75</v>
       </c>
       <c r="D6" t="n">
-        <v>60</v>
+        <v>443</v>
       </c>
       <c r="E6" t="n">
-        <v>60</v>
+        <v>443</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>22.59036445617676</v>
+        <v>516.8385581970215</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m100000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -612,25 +612,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>3.75</v>
       </c>
       <c r="D7" t="n">
-        <v>60</v>
+        <v>443</v>
       </c>
       <c r="E7" t="n">
-        <v>60</v>
+        <v>443</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>12.56886434555054</v>
+        <v>1063.79113984108</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m100000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -639,25 +639,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.25</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>48</v>
+        <v>363</v>
       </c>
       <c r="E8" t="n">
-        <v>48</v>
+        <v>363</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>1.130877494812012</v>
+        <v>872.8907451629639</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m100000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -666,25 +666,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6.25</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>48</v>
+        <v>363</v>
       </c>
       <c r="E9" t="n">
-        <v>48</v>
+        <v>363</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1.699651002883911</v>
+        <v>1222.120064258575</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m100000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -693,25 +693,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5.5</v>
+        <v>4.25</v>
       </c>
       <c r="D10" t="n">
-        <v>102</v>
+        <v>292</v>
       </c>
       <c r="E10" t="n">
-        <v>102</v>
+        <v>292</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>10.46786642074585</v>
+        <v>247.3797736167908</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m100000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -720,25 +720,25 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5.5</v>
+        <v>4.25</v>
       </c>
       <c r="D11" t="n">
-        <v>102</v>
+        <v>292</v>
       </c>
       <c r="E11" t="n">
-        <v>102</v>
+        <v>292</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>7.37566351890564</v>
+        <v>1344.663013458252</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -747,25 +747,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5.75</v>
+        <v>3.25</v>
       </c>
       <c r="D12" t="n">
-        <v>86</v>
+        <v>517</v>
       </c>
       <c r="E12" t="n">
-        <v>86</v>
+        <v>517</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>3.364057540893555</v>
+        <v>6.533698797225952</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -774,25 +774,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5.75</v>
+        <v>3.25</v>
       </c>
       <c r="D13" t="n">
-        <v>86</v>
+        <v>517</v>
       </c>
       <c r="E13" t="n">
-        <v>86</v>
+        <v>517</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>5.145659685134888</v>
+        <v>5.941299200057983</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -801,25 +801,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6</v>
+        <v>3.5</v>
       </c>
       <c r="D14" t="n">
-        <v>81</v>
+        <v>408</v>
       </c>
       <c r="E14" t="n">
-        <v>81</v>
+        <v>408</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>19.76316714286804</v>
+        <v>3.251513004302979</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -828,25 +828,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>3.5</v>
       </c>
       <c r="D15" t="n">
-        <v>81</v>
+        <v>408</v>
       </c>
       <c r="E15" t="n">
-        <v>81</v>
+        <v>408</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>13.05497550964355</v>
+        <v>3.995455265045166</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -855,25 +855,25 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6.25</v>
+        <v>3.75</v>
       </c>
       <c r="D16" t="n">
-        <v>81</v>
+        <v>324</v>
       </c>
       <c r="E16" t="n">
-        <v>81</v>
+        <v>324</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>49.48982429504395</v>
+        <v>6.430626153945923</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -882,25 +882,25 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6.25</v>
+        <v>3.75</v>
       </c>
       <c r="D17" t="n">
-        <v>81</v>
+        <v>324</v>
       </c>
       <c r="E17" t="n">
-        <v>81</v>
+        <v>324</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>43.31560659408569</v>
+        <v>10.34433364868164</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -909,25 +909,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
-        <v>73</v>
+        <v>275</v>
       </c>
       <c r="E18" t="n">
-        <v>73</v>
+        <v>275</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0.2098770141601562</v>
+        <v>8.827866315841675</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -936,25 +936,25 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>73</v>
+        <v>275</v>
       </c>
       <c r="E19" t="n">
-        <v>73</v>
+        <v>275</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0.3160197734832764</v>
+        <v>25.08921718597412</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -963,25 +963,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>5.75</v>
+        <v>4.25</v>
       </c>
       <c r="D20" t="n">
-        <v>68</v>
+        <v>238</v>
       </c>
       <c r="E20" t="n">
-        <v>68</v>
+        <v>238</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>0.3922338485717773</v>
+        <v>14.32716274261475</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m10000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -990,19 +990,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5.75</v>
+        <v>4.25</v>
       </c>
       <c r="D21" t="n">
-        <v>68</v>
+        <v>238</v>
       </c>
       <c r="E21" t="n">
-        <v>68</v>
+        <v>238</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>0.4699275493621826</v>
+        <v>8.536463737487793</v>
       </c>
     </row>
     <row r="22">
@@ -1017,19 +1017,19 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>6</v>
+        <v>3.25</v>
       </c>
       <c r="D22" t="n">
-        <v>62</v>
+        <v>550</v>
       </c>
       <c r="E22" t="n">
-        <v>62</v>
+        <v>550</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2963566780090332</v>
+        <v>0.07401800155639648</v>
       </c>
     </row>
     <row r="23">
@@ -1044,19 +1044,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6</v>
+        <v>3.25</v>
       </c>
       <c r="D23" t="n">
-        <v>62</v>
+        <v>550</v>
       </c>
       <c r="E23" t="n">
-        <v>62</v>
+        <v>550</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>0.194378137588501</v>
+        <v>0.07974433898925781</v>
       </c>
     </row>
     <row r="24">
@@ -1071,19 +1071,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>6.25</v>
+        <v>3.5</v>
       </c>
       <c r="D24" t="n">
-        <v>58</v>
+        <v>459</v>
       </c>
       <c r="E24" t="n">
-        <v>58</v>
+        <v>459</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0.5301437377929688</v>
+        <v>0.07510161399841309</v>
       </c>
     </row>
     <row r="25">
@@ -1098,25 +1098,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>6.25</v>
+        <v>3.5</v>
       </c>
       <c r="D25" t="n">
-        <v>58</v>
+        <v>459</v>
       </c>
       <c r="E25" t="n">
-        <v>58</v>
+        <v>459</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>0.5757479667663574</v>
+        <v>0.2010588645935059</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1125,25 +1125,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>5.5</v>
+        <v>3.75</v>
       </c>
       <c r="D26" t="n">
-        <v>69</v>
+        <v>370</v>
       </c>
       <c r="E26" t="n">
-        <v>69</v>
+        <v>370</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>0.330625057220459</v>
+        <v>0.1578612327575684</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1152,25 +1152,25 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5.5</v>
+        <v>3.75</v>
       </c>
       <c r="D27" t="n">
-        <v>69</v>
+        <v>370</v>
       </c>
       <c r="E27" t="n">
-        <v>69</v>
+        <v>370</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0.4671874046325684</v>
+        <v>0.1355557441711426</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1179,25 +1179,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>5.75</v>
+        <v>4</v>
       </c>
       <c r="D28" t="n">
-        <v>64</v>
+        <v>319</v>
       </c>
       <c r="E28" t="n">
-        <v>64</v>
+        <v>319</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0.709552526473999</v>
+        <v>0.6277315616607666</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1206,25 +1206,25 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>5.75</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>64</v>
+        <v>319</v>
       </c>
       <c r="E29" t="n">
-        <v>64</v>
+        <v>319</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>0.3350467681884766</v>
+        <v>0.5064351558685303</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1233,25 +1233,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6</v>
+        <v>4.25</v>
       </c>
       <c r="D30" t="n">
-        <v>61</v>
+        <v>269</v>
       </c>
       <c r="E30" t="n">
-        <v>61</v>
+        <v>269</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>1.247053623199463</v>
+        <v>0.9717035293579102</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1260,25 +1260,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>6</v>
+        <v>4.25</v>
       </c>
       <c r="D31" t="n">
-        <v>61</v>
+        <v>269</v>
       </c>
       <c r="E31" t="n">
-        <v>61</v>
+        <v>269</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>1.645502328872681</v>
+        <v>0.5412757396697998</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m50000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1287,25 +1287,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6.25</v>
+        <v>3.25</v>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>611</v>
       </c>
       <c r="E32" t="n">
-        <v>50</v>
+        <v>611</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>0.2049617767333984</v>
+        <v>120.6096312999725</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m1000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m50000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1314,25 +1314,25 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>6.25</v>
+        <v>3.25</v>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>611</v>
       </c>
       <c r="E33" t="n">
-        <v>50</v>
+        <v>611</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>0.2906296253204346</v>
+        <v>291.7729880809784</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m50000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1341,25 +1341,25 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
       <c r="D34" t="n">
-        <v>90</v>
+        <v>478</v>
       </c>
       <c r="E34" t="n">
-        <v>90</v>
+        <v>478</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>2.195796012878418</v>
+        <v>7.822831392288208</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m50000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1368,25 +1368,25 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
       <c r="D35" t="n">
-        <v>90</v>
+        <v>478</v>
       </c>
       <c r="E35" t="n">
-        <v>90</v>
+        <v>478</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>2.494259834289551</v>
+        <v>16.51130151748657</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m50000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1395,25 +1395,25 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>5.75</v>
+        <v>3.75</v>
       </c>
       <c r="D36" t="n">
-        <v>79</v>
+        <v>373</v>
       </c>
       <c r="E36" t="n">
-        <v>79</v>
+        <v>373</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>0.8484768867492676</v>
+        <v>23.78416275978088</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m50000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1422,25 +1422,25 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>5.75</v>
+        <v>3.75</v>
       </c>
       <c r="D37" t="n">
-        <v>79</v>
+        <v>373</v>
       </c>
       <c r="E37" t="n">
-        <v>79</v>
+        <v>373</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>1.338965654373169</v>
+        <v>51.48590660095215</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m50000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1449,25 +1449,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D38" t="n">
-        <v>76</v>
+        <v>325</v>
       </c>
       <c r="E38" t="n">
-        <v>76</v>
+        <v>325</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>4.361720323562622</v>
+        <v>101.7281475067139</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m50000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1476,25 +1476,25 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D39" t="n">
-        <v>76</v>
+        <v>325</v>
       </c>
       <c r="E39" t="n">
-        <v>76</v>
+        <v>325</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>4.777086734771729</v>
+        <v>127.7861495018005</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m50000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1503,25 +1503,25 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>6.25</v>
+        <v>4.25</v>
       </c>
       <c r="D40" t="n">
-        <v>65</v>
+        <v>284</v>
       </c>
       <c r="E40" t="n">
-        <v>65</v>
+        <v>284</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>0.3341708183288574</v>
+        <v>175.61829829216</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
+          <t>GRID_PSCLP_n100_m50000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1530,25 +1530,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>6.25</v>
+        <v>4.25</v>
       </c>
       <c r="D41" t="n">
-        <v>65</v>
+        <v>284</v>
       </c>
       <c r="E41" t="n">
-        <v>65</v>
+        <v>284</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>0.938326358795166</v>
+        <v>229.8297560214996</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1557,25 +1557,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>5.5</v>
+        <v>3.25</v>
       </c>
       <c r="D42" t="n">
-        <v>84</v>
+        <v>669</v>
       </c>
       <c r="E42" t="n">
-        <v>84</v>
+        <v>669</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>1.779502630233765</v>
+        <v>3.235840797424316</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1584,25 +1584,25 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>5.5</v>
+        <v>3.25</v>
       </c>
       <c r="D43" t="n">
-        <v>84</v>
+        <v>669</v>
       </c>
       <c r="E43" t="n">
-        <v>84</v>
+        <v>669</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>2.901520490646362</v>
+        <v>2.969690084457397</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1611,25 +1611,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>5.75</v>
+        <v>3.5</v>
       </c>
       <c r="D44" t="n">
-        <v>75</v>
+        <v>519</v>
       </c>
       <c r="E44" t="n">
-        <v>75</v>
+        <v>519</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>2.954685926437378</v>
+        <v>4.838692426681519</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1638,25 +1638,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>5.75</v>
+        <v>3.5</v>
       </c>
       <c r="D45" t="n">
-        <v>75</v>
+        <v>519</v>
       </c>
       <c r="E45" t="n">
-        <v>75</v>
+        <v>519</v>
       </c>
       <c r="F45" t="n">
         <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>2.938645839691162</v>
+        <v>5.233616352081299</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1665,25 +1665,25 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>6</v>
+        <v>3.75</v>
       </c>
       <c r="D46" t="n">
-        <v>65</v>
+        <v>417</v>
       </c>
       <c r="E46" t="n">
-        <v>65</v>
+        <v>417</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>4.727549076080322</v>
+        <v>1.841626882553101</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1692,25 +1692,25 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>3.75</v>
       </c>
       <c r="D47" t="n">
-        <v>65</v>
+        <v>417</v>
       </c>
       <c r="E47" t="n">
-        <v>65</v>
+        <v>417</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>3.410742044448853</v>
+        <v>2.275711536407471</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1719,25 +1719,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>6.25</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
-        <v>59</v>
+        <v>330</v>
       </c>
       <c r="E48" t="n">
-        <v>59</v>
+        <v>330</v>
       </c>
       <c r="F48" t="n">
         <v>0</v>
       </c>
       <c r="G48" t="n">
-        <v>2.567535161972046</v>
+        <v>2.152466297149658</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s2</t>
+          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1746,42 +1746,96 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>6.25</v>
+        <v>4</v>
       </c>
       <c r="D49" t="n">
-        <v>59</v>
+        <v>330.0000000001512</v>
       </c>
       <c r="E49" t="n">
-        <v>59</v>
+        <v>330.0000000001512</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>3.616523265838623</v>
+        <v>2.39594554901123</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>GUROBI</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="D50" t="n">
+        <v>277</v>
+      </c>
+      <c r="E50" t="n">
+        <v>277</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" t="n">
+        <v>4.681516170501709</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>GRID_PSCLP_n100_m5000_d1_100_f10_100_s1</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>CPLEX</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="D51" t="n">
+        <v>277</v>
+      </c>
+      <c r="E51" t="n">
+        <v>277</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" t="n">
+        <v>5.02238392829895</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="n">
-        <v>5.875</v>
-      </c>
-      <c r="D50" t="n">
-        <v>70.54166666666667</v>
-      </c>
-      <c r="E50" t="n">
-        <v>70.54166666666667</v>
-      </c>
-      <c r="F50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" t="n">
-        <v>5.823189770181973</v>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D52" t="n">
+        <v>414.8800000000031</v>
+      </c>
+      <c r="E52" t="n">
+        <v>414.8800000000031</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
+        <v>169.772534661293</v>
       </c>
     </row>
   </sheetData>

</xml_diff>